<commit_message>
Finalized setup for triple2text
</commit_message>
<xml_diff>
--- a/evaluation/evaluation.xlsx
+++ b/evaluation/evaluation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramaw\Documents\master-thesis\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA7C0003-CC7D-4DFA-9AB7-6B72CA150791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647D995E-F1DA-4107-B10B-DC137B0AADE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{72E58FE3-2FF7-4DAF-898B-173E722938DB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{72E58FE3-2FF7-4DAF-898B-173E722938DB}"/>
   </bookViews>
   <sheets>
     <sheet name="text2sparql-A-8B" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="75">
   <si>
     <t>id</t>
   </si>
@@ -296,6 +296,9 @@
   </si>
   <si>
     <t>exact query as A70B</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -2033,13 +2036,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G21" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H21" s="1" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+      <c r="G21" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>74</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="3"/>
@@ -2557,7 +2558,7 @@
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -2791,13 +2792,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="G21" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H21" s="1" t="e">
-        <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+      <c r="G21" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>74</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="3"/>

</xml_diff>